<commit_message>
Intégration des Modèles Métier des sections+entrées ee744eba2fe5e450e05c2f13b74fe0839fa9485c
</commit_message>
<xml_diff>
--- a/htr-Corps-ModeleMetier/ig/StructureDefinition-AllergiesEtHypersensibilites.xlsx
+++ b/htr-Corps-ModeleMetier/ig/StructureDefinition-AllergiesEtHypersensibilites.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="100">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-05-27T14:36:02+00:00</t>
+    <t>2025-06-05T15:38:56+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -292,30 +292,26 @@
     <t>AllergiesEtHypersensibilites.sousSection</t>
   </si>
   <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/Section
-</t>
-  </si>
-  <si>
-    <t>Sous-sections</t>
-  </si>
-  <si>
-    <t>Section.sousSection</t>
-  </si>
-  <si>
-    <t>AllergiesEtHypersensibilites.entree</t>
-  </si>
-  <si>
     <t xml:space="preserve">Base
 </t>
   </si>
   <si>
+    <t>Sous-sections</t>
+  </si>
+  <si>
+    <t>Section.sousSection</t>
+  </si>
+  <si>
+    <t>AllergiesEtHypersensibilites.entree</t>
+  </si>
+  <si>
     <t>Entrées</t>
   </si>
   <si>
     <t>Section.entree</t>
   </si>
   <si>
-    <t>AllergiesEtHypersensibilites.allergieOuHypersensibilite</t>
+    <t>AllergiesEtHypersensibilites.entree.allergieOuHypersensibilite</t>
   </si>
   <si>
     <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/AllergieOuHypersensibilite
@@ -627,8 +623,8 @@
   <dimension ref="A1:AJ8"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="43.9921875" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="43.9921875" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="49.65234375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="49.65234375" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="7.6796875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
@@ -658,7 +654,7 @@
     <col min="29" max="29" width="17.65625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="32" max="32" width="43.9921875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="32" max="32" width="49.65234375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
@@ -1190,7 +1186,7 @@
         <v>73</v>
       </c>
       <c r="G6" t="s" s="2">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H6" t="s" s="2">
         <v>72</v>
@@ -1287,7 +1283,7 @@
       </c>
       <c r="E7" s="2"/>
       <c r="F7" t="s" s="2">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="G7" t="s" s="2">
         <v>74</v>
@@ -1302,13 +1298,13 @@
         <v>72</v>
       </c>
       <c r="K7" t="s" s="2">
+        <v>91</v>
+      </c>
+      <c r="L7" t="s" s="2">
         <v>95</v>
       </c>
-      <c r="L7" t="s" s="2">
-        <v>96</v>
-      </c>
       <c r="M7" t="s" s="2">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
@@ -1359,7 +1355,7 @@
         <v>72</v>
       </c>
       <c r="AF7" t="s" s="2">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="AG7" t="s" s="2">
         <v>73</v>
@@ -1376,10 +1372,10 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
@@ -1402,13 +1398,13 @@
         <v>72</v>
       </c>
       <c r="K8" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="L8" t="s" s="2">
         <v>99</v>
       </c>
-      <c r="L8" t="s" s="2">
-        <v>100</v>
-      </c>
       <c r="M8" t="s" s="2">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
@@ -1459,7 +1455,7 @@
         <v>72</v>
       </c>
       <c r="AF8" t="s" s="2">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="AG8" t="s" s="2">
         <v>78</v>

</xml_diff>